<commit_message>
fix lỗi trướng bị chiếu
</commit_message>
<xml_diff>
--- a/Extra/tasks/Phân Công_Tuần 4.xlsx
+++ b/Extra/tasks/Phân Công_Tuần 4.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\UTH mãi đỉnh\Lập trình Mạng\Project\NET_09-CO-TUONG\Extra\tasks\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{E692F186-749B-4600-8797-275565235A11}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{206B49CB-50CA-40CE-B8CA-C3A5FEBB540E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -31,15 +31,9 @@
     <t>Sản phẩm cuối cùng</t>
   </si>
   <si>
-    <t>Server ổn định 24/7</t>
-  </si>
-  <si>
     <t>ConnectionGuard.cs</t>
   </si>
   <si>
-    <t>Giao diện hoàn chỉnh</t>
-  </si>
-  <si>
     <t>FinalLogic.cs</t>
   </si>
   <si>
@@ -86,6 +80,12 @@
   </si>
   <si>
     <t>Nhiệm vụ chi tiết</t>
+  </si>
+  <si>
+    <t>SoundManager.cs</t>
+  </si>
+  <si>
+    <t>Server ổn định</t>
   </si>
 </sst>
 </file>
@@ -426,7 +426,7 @@
         <v>1</v>
       </c>
       <c r="C1" s="4" t="s">
-        <v>21</v>
+        <v>19</v>
       </c>
       <c r="D1" s="4" t="s">
         <v>2</v>
@@ -437,13 +437,13 @@
         <v>1</v>
       </c>
       <c r="B2" s="2" t="s">
-        <v>9</v>
+        <v>7</v>
       </c>
       <c r="C2" s="5" t="s">
-        <v>18</v>
+        <v>16</v>
       </c>
       <c r="D2" s="1" t="s">
-        <v>3</v>
+        <v>21</v>
       </c>
     </row>
     <row r="3" spans="1:4" ht="30" customHeight="1" x14ac:dyDescent="0.25">
@@ -451,13 +451,13 @@
         <v>2</v>
       </c>
       <c r="B3" s="2" t="s">
-        <v>10</v>
+        <v>8</v>
       </c>
       <c r="C3" s="5" t="s">
-        <v>19</v>
+        <v>17</v>
       </c>
       <c r="D3" s="1" t="s">
-        <v>4</v>
+        <v>3</v>
       </c>
     </row>
     <row r="4" spans="1:4" ht="32.25" customHeight="1" x14ac:dyDescent="0.25">
@@ -465,13 +465,13 @@
         <v>3</v>
       </c>
       <c r="B4" s="2" t="s">
-        <v>11</v>
+        <v>9</v>
       </c>
       <c r="C4" s="5" t="s">
-        <v>15</v>
+        <v>13</v>
       </c>
       <c r="D4" s="1" t="s">
-        <v>5</v>
+        <v>20</v>
       </c>
     </row>
     <row r="5" spans="1:4" ht="33.75" customHeight="1" x14ac:dyDescent="0.25">
@@ -479,13 +479,13 @@
         <v>4</v>
       </c>
       <c r="B5" s="2" t="s">
-        <v>12</v>
+        <v>10</v>
       </c>
       <c r="C5" s="5" t="s">
-        <v>16</v>
+        <v>14</v>
       </c>
       <c r="D5" s="1" t="s">
-        <v>6</v>
+        <v>4</v>
       </c>
     </row>
     <row r="6" spans="1:4" ht="32.25" customHeight="1" x14ac:dyDescent="0.25">
@@ -493,13 +493,13 @@
         <v>5</v>
       </c>
       <c r="B6" s="2" t="s">
-        <v>13</v>
+        <v>11</v>
       </c>
       <c r="C6" s="5" t="s">
-        <v>20</v>
+        <v>18</v>
       </c>
       <c r="D6" s="1" t="s">
-        <v>7</v>
+        <v>5</v>
       </c>
     </row>
     <row r="7" spans="1:4" ht="30.75" customHeight="1" x14ac:dyDescent="0.25">
@@ -507,13 +507,13 @@
         <v>6</v>
       </c>
       <c r="B7" s="2" t="s">
-        <v>14</v>
+        <v>12</v>
       </c>
       <c r="C7" s="5" t="s">
-        <v>17</v>
+        <v>15</v>
       </c>
       <c r="D7" s="1" t="s">
-        <v>8</v>
+        <v>6</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
sửa task và xóa file
</commit_message>
<xml_diff>
--- a/Extra/tasks/Phân Công_Tuần 4.xlsx
+++ b/Extra/tasks/Phân Công_Tuần 4.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30430"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30527"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\UTH mãi đỉnh\Lập trình Mạng\Project\NET_09-CO-TUONG\Extra\tasks\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{206B49CB-50CA-40CE-B8CA-C3A5FEBB540E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{1B596A4D-A953-4FDB-951F-EF0898A5CD2D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -20,7 +20,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="22" uniqueCount="22">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="22" uniqueCount="17">
   <si>
     <t>STT</t>
   </si>
@@ -31,18 +31,6 @@
     <t>Sản phẩm cuối cùng</t>
   </si>
   <si>
-    <t>ConnectionGuard.cs</t>
-  </si>
-  <si>
-    <t>FinalLogic.cs</t>
-  </si>
-  <si>
-    <t>GameTimer.cs</t>
-  </si>
-  <si>
-    <t>ChatHandler.cs</t>
-  </si>
-  <si>
     <t>Trần Nhật Sinh</t>
   </si>
   <si>
@@ -67,25 +55,22 @@
     <t>Fix lỗi logic di chuyển &amp; các trường hợp đặc biệt.</t>
   </si>
   <si>
-    <t>Code chung: Chat, Login &amp; Chạy Stress Test hệ thống.</t>
-  </si>
-  <si>
     <t xml:space="preserve"> Demo toàn bộ tính năng. Tối ưu Server.</t>
   </si>
   <si>
-    <t>Xử lý Auto-reconnect &amp; Phụ làm Login.</t>
-  </si>
-  <si>
-    <t>Đồng bộ Timer &amp; Phụ làm Giao thức Chat.</t>
-  </si>
-  <si>
     <t>Nhiệm vụ chi tiết</t>
   </si>
   <si>
-    <t>SoundManager.cs</t>
-  </si>
-  <si>
-    <t>Server ổn định</t>
+    <t>Xử lý Auto-reconnect</t>
+  </si>
+  <si>
+    <t>Đồng bộ Timer</t>
+  </si>
+  <si>
+    <t>Chat, Login &amp; Chạy Stress Test hệ thống.</t>
+  </si>
+  <si>
+    <t>Hoàn thành code</t>
   </si>
 </sst>
 </file>
@@ -414,7 +399,7 @@
   <cols>
     <col min="1" max="1" width="7" customWidth="1"/>
     <col min="2" max="2" width="19.88671875" customWidth="1"/>
-    <col min="3" max="3" width="121.33203125" customWidth="1"/>
+    <col min="3" max="3" width="73.33203125" customWidth="1"/>
     <col min="4" max="4" width="22.77734375" customWidth="1"/>
   </cols>
   <sheetData>
@@ -426,7 +411,7 @@
         <v>1</v>
       </c>
       <c r="C1" s="4" t="s">
-        <v>19</v>
+        <v>12</v>
       </c>
       <c r="D1" s="4" t="s">
         <v>2</v>
@@ -437,13 +422,13 @@
         <v>1</v>
       </c>
       <c r="B2" s="2" t="s">
-        <v>7</v>
+        <v>3</v>
       </c>
       <c r="C2" s="5" t="s">
+        <v>11</v>
+      </c>
+      <c r="D2" s="1" t="s">
         <v>16</v>
-      </c>
-      <c r="D2" s="1" t="s">
-        <v>21</v>
       </c>
     </row>
     <row r="3" spans="1:4" ht="30" customHeight="1" x14ac:dyDescent="0.25">
@@ -451,13 +436,13 @@
         <v>2</v>
       </c>
       <c r="B3" s="2" t="s">
-        <v>8</v>
+        <v>4</v>
       </c>
       <c r="C3" s="5" t="s">
-        <v>17</v>
+        <v>13</v>
       </c>
       <c r="D3" s="1" t="s">
-        <v>3</v>
+        <v>16</v>
       </c>
     </row>
     <row r="4" spans="1:4" ht="32.25" customHeight="1" x14ac:dyDescent="0.25">
@@ -465,13 +450,13 @@
         <v>3</v>
       </c>
       <c r="B4" s="2" t="s">
+        <v>5</v>
+      </c>
+      <c r="C4" s="5" t="s">
         <v>9</v>
       </c>
-      <c r="C4" s="5" t="s">
-        <v>13</v>
-      </c>
       <c r="D4" s="1" t="s">
-        <v>20</v>
+        <v>16</v>
       </c>
     </row>
     <row r="5" spans="1:4" ht="33.75" customHeight="1" x14ac:dyDescent="0.25">
@@ -479,13 +464,13 @@
         <v>4</v>
       </c>
       <c r="B5" s="2" t="s">
+        <v>6</v>
+      </c>
+      <c r="C5" s="5" t="s">
         <v>10</v>
       </c>
-      <c r="C5" s="5" t="s">
-        <v>14</v>
-      </c>
       <c r="D5" s="1" t="s">
-        <v>4</v>
+        <v>16</v>
       </c>
     </row>
     <row r="6" spans="1:4" ht="32.25" customHeight="1" x14ac:dyDescent="0.25">
@@ -493,13 +478,13 @@
         <v>5</v>
       </c>
       <c r="B6" s="2" t="s">
-        <v>11</v>
+        <v>7</v>
       </c>
       <c r="C6" s="5" t="s">
-        <v>18</v>
+        <v>14</v>
       </c>
       <c r="D6" s="1" t="s">
-        <v>5</v>
+        <v>16</v>
       </c>
     </row>
     <row r="7" spans="1:4" ht="30.75" customHeight="1" x14ac:dyDescent="0.25">
@@ -507,13 +492,13 @@
         <v>6</v>
       </c>
       <c r="B7" s="2" t="s">
-        <v>12</v>
+        <v>8</v>
       </c>
       <c r="C7" s="5" t="s">
         <v>15</v>
       </c>
       <c r="D7" s="1" t="s">
-        <v>6</v>
+        <v>16</v>
       </c>
     </row>
   </sheetData>

</xml_diff>